<commit_message>
feat(pipeline): complete 10 Portuguese Sardinhas designs, mockups, Printify 8/20 config, Etsy sync, and Pinterest export
</commit_message>
<xml_diff>
--- a/CaseCraft_Pinterest_Single_Mockup.xlsx
+++ b/CaseCraft_Pinterest_Single_Mockup.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -517,12 +517,12 @@
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Surreal Suncatcher Vitrail Mini Frog Floating Lava Lamp Tough Case</t>
+          <t>The Porto Classic Sardinhas in Olive Oil Tough Phone Case</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261012133501-1f1c641b-96f5-69c8-9f99-7ae38c3b7b9e.png</t>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104255-1f1c6f2d-8fb1-6f1e-9440-7e9a5149d519.png</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -533,34 +533,34 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Surreal stained glass vitrail suncatcher phone case featuring an adorable mini green frog floating peacefully inside a glowing molten lava lamp under rainbow prism light. Dual-layer impact-resistant polycarbonate outer shell with shock-absorbing TPU inner liner. Fits 34 iPhone &amp; Samsung Galaxy models.</t>
+          <t>Iconic Porto classic canned sardines in pure golden olive oil framed by ornate handcrafted blue-and-white Portuguese Baroque Azulejo ceramic tiles, fresh Mediterranean lemon slices, and olive sprigs. Premium dual-layer Tough Case with impact-resistant polycarbonate backplate.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=suncatcher_frog_002</t>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-001</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>suncatcher frog, vitrail phone case, floating frog case, lava lamp case, stained glass frog, cute frog phone case, iphone 18 pro max, samsung galaxy s26, tough phone case, rainbow prism case, groovy retro frog, cottagecore frog, frog lover gift</t>
+          <t>portuguese sardines, porto azulejo case, sardinhas case, blue tile phone case, portugal travel gift, lisbon souvenir, azulejo tile art, olive oil sardine, vintage tin case, iphone 18 pro max, samsung galaxy s26, tough phone case, mediterranean art</t>
         </is>
       </c>
     </row>
     <row r="3" ht="54" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Gothic Cathedral Vitrail Wizard Frog Lava Potion Lamp Tough Case</t>
+          <t>Galo de Barcelos Portuguese Rooster Spicy Sardines Tough Case</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261012133905-1f1c6424-ae2e-6ec4-904c-1ee442ad1e48.png</t>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104338-1f1c6f2f-3248-6862-91aa-4eb37dd39630.png</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -571,34 +571,34 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Gothic cathedral stained glass vitrail phone case featuring a wise wizard frog in a celestial purple hat holding a crystal staff beside a bubbling molten lava potion lamp beneath cathedral rose windows. Premium dual-layer Tough Case with impact-resistant polycarbonate outer shell.</t>
+          <t>Traditional Portuguese folk art Galo de Barcelos lucky rooster perched proudly atop a vintage crimson sardine tin with fiery piri-piri chili peppers, hearts, and floral motifs. Dual-layer shock-absorbing Tough Case.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=wizard_frog_003</t>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-002</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>wizard frog case, gothic stained glass, vitrail phone case, potion lava lamp, witchy frog case, cathedral vitrail, iphone 18 pro max, samsung galaxy s26, tough phone case, dark academia frog, fantasy frog cover, cottagecore witch, magical frog gift</t>
+          <t>galo de barcelos, portuguese rooster, piri piri sardines, portugal folk art, spicy sardine case, barcelos rooster, lisbon souvenir, iphone 18 pro max, samsung galaxy s26, tough phone case, portuguese gift, retro tin can, portugal pride</t>
         </is>
       </c>
     </row>
     <row r="4" ht="54" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Celestial Tarot Card Vitrail Moon Frog Sacred Lava Lamp Tough Case</t>
+          <t>Algarve Coastal Fisherman Morning Haul Sardines Tough Case</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261012133954-1f1c6426-811f-603a-a834-2a95200fac38.png</t>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104423-1f1c6f30-d94b-6578-a698-8a1193b0d0c8.png</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -609,34 +609,34 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Celestial tarot card stained glass vitrail phone case featuring a mystical moon frog perched on a golden crescent moon beside a glowing sacred lava lamp under midnight constellations and luna moths. Premium dual-layer Tough Case with shock-absorbing TPU liner.</t>
+          <t>Vintage maritime nautical woodcut illustration of a weathered Portuguese fisherman in a traditional barrete wool cap hauling shimmering silver Atlantic sardines into a rustic coastal tin. Heavy-duty dual-layer Tough Case.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=tarot_frog_004</t>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-003</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>celestial tarot case, moon frog case, vitrail phone case, stained glass moon, sacred lava lamp, tarot card case, iphone 18 pro max, samsung galaxy s26, tough phone case, luna moth case, witchy aesthetic, mystical frog gift, zodiac phone case</t>
+          <t>algarve fisherman, nautical phone case, sardine haul tin, portugal coast art, atlantic sardines, fisherman gift, vintage maritime, iphone 18 pro max, samsung galaxy s26, tough phone case, ocean beach case, portuguese sea art, coastal decor</t>
         </is>
       </c>
     </row>
     <row r="5" ht="54" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Western Disco Vitrail 70s Cowboy Frog Desert Lava Lamp Tough Case</t>
+          <t>Fado Night Sardinhas and Portuguese Guitar Tough Phone Case</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261012134043-1f1c6428-58bb-654c-891e-16ec86c827dd.png</t>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104508-1f1c6f32-8654-6354-8b6e-a6efca640832.png</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -647,34 +647,34 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Western disco 1970s stained glass vitrail phone case featuring a groovy cowboy frog in a ten-gallon Stetson hat under a sparkling disco ball beside a desert saguaro cactus lava lamp. Impact-resistant dual-layer Tough Case with glossy vibrant backplate.</t>
+          <t>Atmospheric midnight lithograph featuring a traditional 12-string Guitarra Portuguesa resting against an open vintage sardine tin in the cobbled lantern-lit alleyways of Alfama Lisbon. Protective dual-layer Tough Case.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=cowboy_frog_005</t>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-004</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>cowboy frog case, western disco case, 70s retro vitrail, desert lava lamp, stained glass frog, disco cowgirl case, iphone 18 pro max, samsung galaxy s26, tough phone case, country western frog, groovy 70s case, yall frog gift, rodeo frog cover</t>
+          <t>fado music case, guitarra portuguesa, alfama lisbon case, fado night sardines, portuguese guitar, lisbon fado gift, midnight lithograph, iphone 18 pro max, samsung galaxy s26, tough phone case, portugal music lover, romantic lisbon, vintage fado</t>
         </is>
       </c>
     </row>
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>70s Vinyl Lo-Fi DJ Frog Bubbling Lava Lamp Vitrail Tough Case</t>
+          <t>Tram 28 Lisbon Sardine Express Vintage Travel Tough Case</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261012134129-1f1c642a-121e-6326-baa6-32424d5077df.png</t>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104552-1f1c6f34-2dc1-6f00-8967-7290343d7267.png</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -685,34 +685,34 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Chill lo-fi 1970s stained glass vitrail phone case featuring a retro audiophile DJ frog wearing gold headphones spinning vintage vinyl on a turntable beside a bubbling warm amber lava lamp. Dual-layer shock-absorbing protective Tough Case.</t>
+          <t>Vintage European travel poster styling showcasing the iconic yellow Lisbon Tram 28 reimagined as a retro Sardinhas de Lisboa tin gliding over sunlit Portuguese cobblestone streets. Durable dual-layer Tough Case.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=lofi_frog_006</t>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-005</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>lofi frog case, dj frog phone case, vinyl record case, 70s audio vitrail, bubbling lava lamp, retro audiophile, iphone 18 pro max, samsung galaxy s26, tough phone case, chill lofi hip hop, stained glass frog, music lover gift, turntable case</t>
+          <t>tram 28 lisbon, yellow tram case, sardinhas de lisboa, lisbon travel poster, portugal wanderlust, vintage travel tin, tram 28 souvenir, iphone 18 pro max, samsung galaxy s26, tough phone case, lisbon city case, european traveler, street tram art</t>
         </is>
       </c>
     </row>
     <row r="7" ht="54" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>UV Blacklight Cyber-Vitrail Acid-Melt Lava Lamp Frog Tough Case</t>
+          <t>Azulejo Tile Mosaic Silver Pilchard Trio Tough Phone Case</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261012134216-1f1c642b-d1cf-6426-874a-32424d5077df.png</t>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104637-1f1c6f35-d7cd-6aca-abdf-7290343d7267.png</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -723,22 +723,174 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Electric neon UV blacklight psychedelic cyber-vitrail phone case featuring an acid-melt trippy cyber frog bathed in glowing fluorescent magenta, electric cyan, and neon green lava droplets. Dual-layer ultra-durable Tough Case.</t>
+          <t>Harmonious circular Yin-Yang swimming medallion of three sleek silver sardines set in an authentic cobalt-blue and white geometric Portuguese Azulejo ceramic tile mosaic. Dual-layer impact-resistant Tough Case.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=cyber_frog_007</t>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-006</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>uv blacklight case, cyber vitrail case, neon frog case, acid melt lava lamp, psychedelic phone cover, trippy rave case, iphone 18 pro max, samsung galaxy s26, tough phone case, fluorescent frog, edm rave aesthetic, electric neon case, cyberpunk frog</t>
+          <t>azulejo tile mosaic, silver sardines case, pilchard trio art, portuguese ceramic, delft blue tile, yinyang fish case, minimalist tile art, iphone 18 pro max, samsung galaxy s26, tough phone case, mediterranean tile, lisbon aesthetic, geometric fish</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Belem Tower Maritime Sardine Cannery Label Tough Case</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104721-1f1c6f37-8127-67d2-a1a5-8a1193b0d0c8.png</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>19th-century royal archival engraving of Lisbon's historic Torre de Belém fortress framed by the Portuguese royal coat of arms, maritime armillary spheres, and vintage Conservas Reais typography. Tough Case.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-007</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>belem tower case, torre de belem, conservas reais, royal sardine tin, portugal history art, vintage engraving, lisbon monument, iphone 18 pro max, samsung galaxy s26, tough phone case, archival travel case, architecture lover, portuguese empire</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sardinha com Pimentos Grilled Pepper Sardine Fest Tough Case</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104806-1f1c6f39-2bce-65d6-a928-4eb37dd39630.png</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Sizzling Santos Populares street festival celebration featuring charred grilled sardines served over rustic broa cornbread with charred red and green bell peppers and summer festival garland. Durable Tough Case.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-008</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>sardinha com pimentos, grilled sardines, santos populares, festa de lisboa, portuguese food art, sardine festival, broa cornbread, iphone 18 pro max, samsung galaxy s26, tough phone case, foodie phone case, portugal summer fest, lisbon street food</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Madeira Island Exotic Passion Fruit Sardine Tough Case</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104850-1f1c6f3a-d0c9-6972-917c-c6926db4fc70.png</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Botanical Art Nouveau vintage sardine tin label adorned with exotic Madeira passion fruit blossoms, lush banana leaves, and rugged Atlantic volcanic cliffs. Protective dual-layer Tough Case.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-009</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>madeira island case, passion fruit tin, botanical art nouveau, tropical sardine, portugal islands, madeira flower fest, atlantic island art, iphone 18 pro max, samsung galaxy s26, tough phone case, funchal souvenir, exotic botanical, volcanic cliffs</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Cascais Riviera Sunbather Sardine Picnic Tough Case</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104935-1f1c6f3c-79c2-680c-9a78-a6efca640832.png</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Chic 1950s Mid-Century French-Portuguese Riviera gouache featuring cat-eye sunglasses, striped beach cabana umbrella, and a golden sardine tin on a sun-drenched Cascais sandy beach towel. Dual-layer Tough Case.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-010</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>cascais riviera, beach picnic case, retro sunbather, mid century gouache, portugal beach case, coastal summer tin, vintage 1950s resort, iphone 18 pro max, samsung galaxy s26, tough phone case, summer vacation gift, estoril coast, sandy beach picnic</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix phone case mockups: zero overflow, exact boundaries, updated Printify & Etsy listings
</commit_message>
<xml_diff>
--- a/CaseCraft_Pinterest_Single_Mockup.xlsx
+++ b/CaseCraft_Pinterest_Single_Mockup.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pinterest_Single_Mockup" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pinterest Pins" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,24 +26,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <color rgb="00111827"/>
+      <name val="Segoe UI"/>
+      <color rgb="001F2937"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="001D4ED8"/>
-      <sz val="10"/>
-      <u val="single"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -52,8 +46,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E60023"/>
-        <bgColor rgb="00E60023"/>
+        <fgColor rgb="00111827"/>
+        <bgColor rgb="00111827"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9FAFB"/>
+        <bgColor rgb="00F9FAFB"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,32 +67,38 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="00E5E7EB"/>
       </left>
       <right style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="00E5E7EB"/>
       </right>
       <top style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="00E5E7EB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="00E5E7EB"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,20 +465,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="75" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="64" customWidth="1" min="5" max="5"/>
-    <col width="65" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Title</t>
@@ -514,383 +520,649 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="54" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Stained Glass Frog Phone Case | Tough Phone Case</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013125521-1f1c7055-97dc-63d2-b125-0242e9a27744.png</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bring a little wonder to everyday moments with this vibrant phone case. The stained-glass–inspired artwork features a chill, bespectacled frog lounging among mushrooms and a glowing lava lamp—warm amber light pouring down like sunset through a cozy window. The scene feels like a tucked-away living room in the woods: relaxed, slightly retro, and full of small, silly magic. This case wears the artwork like a miniature poster, turning your device into something playful you’ll enjoy seeing all </t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>frog phone case, stained glass case, tough phone case, aesthetic frog case, vitrail art, retro lava lamp case</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Surreal Suncatcher Vitrail Mini Frog Floating Lava Lamp Tough Case</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013125557-1f1c7056-ebe0-6798-84b3-ea2cf2970eba.png</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Surreal stained glass vitrail suncatcher phone case featuring an adorable mini green frog floating peacefully inside a glowing molten lava lamp under rainbow prism light. Dual-layer impact-resistant polycarbonate outer shell with shock-absorbing TPU inner liner.</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>suncatcher frog case, mini frog lava lamp, vitrail phone case, cute frog phone case, psychedelic phone case, iphone 18 case</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Gothic Cathedral Vitrail Wizard Frog Lava Potion Lamp Tough Case</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013125635-1f1c7058-5a97-6fdc-a976-ea2cf2970eba.png</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Gothic cathedral stained glass vitrail phone case featuring a wise wizard frog in a celestial purple hat holding a crystal staff beside a bubbling molten lava potion lamp beneath cathedral rose windows. Premium dual-layer Tough Case with impact-resistant polycarbonate outer shell.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>gothic wizard frog case, potion bottle phone case, stained glass gothic case, fantasy frog case, dark academia phone case</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Celestial Tarot Card Vitrail Moon Frog Sacred Lava Lamp Tough Case</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013125715-1f1c7059-d904-6054-a71a-8a1c52550bdc.png</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Celestial tarot card stained glass vitrail phone case featuring a mystical moon frog perched on a golden crescent moon beside a glowing sacred lava lamp under midnight constellations and luna moths. Premium dual-layer Tough Case with shock-absorbing TPU liner.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>celestial tarot frog case, moon frog phone case, mystic lava lamp case, occult vitrail case, galaxy frog tough case</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Western Disco Vitrail 70s Cowboy Frog Desert Lava Lamp Tough Case</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013125755-1f1c705b-518f-6b76-beab-a6efca640832.png</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Western disco 1970s stained glass vitrail phone case featuring a groovy cowboy frog in a ten-gallon Stetson hat under a sparkling disco ball beside a desert saguaro cactus lava lamp. Impact-resistant dual-layer Tough Case with glossy vibrant backplate.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>western cowboy frog case, disco lava lamp phone case, 70s retro phone case, desert frog case, boho western case</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>70s Vinyl Lo-Fi DJ Frog Bubbling Lava Lamp Vitrail Tough Case</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013125835-1f1c705c-d05e-6384-bcce-ea2cf2970eba.png</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Chill lo-fi 1970s stained glass vitrail phone case featuring a retro audiophile DJ frog wearing gold headphones spinning vintage vinyl on a turntable beside a bubbling warm amber lava lamp. Dual-layer shock-absorbing protective Tough Case.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>lofi dj frog case, 70s vinyl phone case, bubbling lava lamp case, aesthetic music phone case, cute dj frog cover</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>UV Blacklight Cyber-Vitrail Acid-Melt Lava Lamp Frog Tough Case</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013125915-1f1c705e-4eaa-6458-8998-a6efca640832.png</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Electric neon UV blacklight psychedelic cyber-vitrail phone case featuring an acid-melt trippy cyber frog bathed in glowing fluorescent magenta, electric cyan, and neon green lava droplets. Dual-layer ultra-durable Tough Case.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>uv blacklight frog case, cyber vitrail case, acid melt lava lamp case, neon frog phone case, vaporwave phone case</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>The Porto Classic Sardinhas in Olive Oil Tough Phone Case</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104255-1f1c6f2d-8fb1-6f1e-9440-7e9a5149d519.png</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013125954-1f1c705f-c132-6024-b2f1-a6efca640832.png</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Iconic Porto classic canned sardines in pure golden olive oil framed by ornate handcrafted blue-and-white Portuguese Baroque Azulejo ceramic tiles, fresh Mediterranean lemon slices, and olive sprigs. Premium dual-layer Tough Case with impact-resistant polycarbonate backplate.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-001</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>portuguese sardines, porto azulejo case, sardinhas case, blue tile phone case, portugal travel gift, lisbon souvenir, azulejo tile art, olive oil sardine, vintage tin case, iphone 18 pro max, samsung galaxy s26, tough phone case, mediterranean art</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="54" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>portuguese sardine case, porto classic sardines, azulejo tile phone case, olive oil tin case, portugal souvenir case</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Galo de Barcelos Portuguese Rooster Spicy Sardines Tough Case</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104338-1f1c6f2f-3248-6862-91aa-4eb37dd39630.png</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013130033-1f1c7061-3a2b-66aa-9020-8a1c52550bdc.png</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Traditional Portuguese folk art Galo de Barcelos lucky rooster perched proudly atop a vintage crimson sardine tin with fiery piri-piri chili peppers, hearts, and floral motifs. Dual-layer shock-absorbing Tough Case.</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-002</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>galo de barcelos, portuguese rooster, piri piri sardines, portugal folk art, spicy sardine case, barcelos rooster, lisbon souvenir, iphone 18 pro max, samsung galaxy s26, tough phone case, portuguese gift, retro tin can, portugal pride</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="54" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>galo de barcelos case, portuguese rooster phone case, spicy sardine case, piri piri phone case, portuguese folk art case</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Algarve Coastal Fisherman Morning Haul Sardines Tough Case</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104423-1f1c6f30-d94b-6578-a698-8a1193b0d0c8.png</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013130112-1f1c7062-a90c-6082-b1a1-c6926db4fc70.png</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Vintage maritime nautical woodcut illustration of a weathered Portuguese fisherman in a traditional barrete wool cap hauling shimmering silver Atlantic sardines into a rustic coastal tin. Heavy-duty dual-layer Tough Case.</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-003</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>algarve fisherman, nautical phone case, sardine haul tin, portugal coast art, atlantic sardines, fisherman gift, vintage maritime, iphone 18 pro max, samsung galaxy s26, tough phone case, ocean beach case, portuguese sea art, coastal decor</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="54" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>algarve fisherman case, vintage nautical phone case, sardine haul tin case, portugal beach phone case, sea lover tough case</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Fado Night Sardinhas and Portuguese Guitar Tough Phone Case</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104508-1f1c6f32-8654-6354-8b6e-a6efca640832.png</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013132449-1f1c7097-7175-6c4c-97ad-d6a35634e85c.png</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Atmospheric midnight lithograph featuring a traditional 12-string Guitarra Portuguesa resting against an open vintage sardine tin in the cobbled lantern-lit alleyways of Alfama Lisbon. Protective dual-layer Tough Case.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-004</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>fado music case, guitarra portuguesa, alfama lisbon case, fado night sardines, portuguese guitar, lisbon fado gift, midnight lithograph, iphone 18 pro max, samsung galaxy s26, tough phone case, portugal music lover, romantic lisbon, vintage fado</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="54" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>fado guitar phone case, alfama lisbon phone case, sardinha fado case, romantic portugal case, vintage midnight tin case</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Tram 28 Lisbon Sardine Express Vintage Travel Tough Case</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104552-1f1c6f34-2dc1-6f00-8967-7290343d7267.png</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013132521-1f1c7098-a7ac-66ac-a537-a6efca640832.png</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Vintage European travel poster styling showcasing the iconic yellow Lisbon Tram 28 reimagined as a retro Sardinhas de Lisboa tin gliding over sunlit Portuguese cobblestone streets. Durable dual-layer Tough Case.</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-005</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>tram 28 lisbon, yellow tram case, sardinhas de lisboa, lisbon travel poster, portugal wanderlust, vintage travel tin, tram 28 souvenir, iphone 18 pro max, samsung galaxy s26, tough phone case, lisbon city case, european traveler, street tram art</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="54" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>tram 28 lisbon case, yellow tram phone case, sardinhas de lisboa case, portugal travel poster case, vintage tram case</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Azulejo Tile Mosaic Silver Pilchard Trio Tough Phone Case</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104637-1f1c6f35-d7cd-6aca-abdf-7290343d7267.png</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013132555-1f1c7099-e63a-688c-a71f-8a1c52550bdc.png</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Harmonious circular Yin-Yang swimming medallion of three sleek silver sardines set in an authentic cobalt-blue and white geometric Portuguese Azulejo ceramic tile mosaic. Dual-layer impact-resistant Tough Case.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-006</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>azulejo tile mosaic, silver sardines case, pilchard trio art, portuguese ceramic, delft blue tile, yinyang fish case, minimalist tile art, iphone 18 pro max, samsung galaxy s26, tough phone case, mediterranean tile, lisbon aesthetic, geometric fish</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="54" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>azulejo tile mosaic case, silver pilchard phone case, blue white ceramic tile case, delft tile phone case, portuguese tile case</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Belem Tower Maritime Sardine Cannery Label Tough Case</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104721-1f1c6f37-8127-67d2-a1a5-8a1193b0d0c8.png</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>19th-century royal archival engraving of Lisbon's historic Torre de Belém fortress framed by the Portuguese royal coat of arms, maritime armillary spheres, and vintage Conservas Reais typography. Tough Case.</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-007</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>belem tower case, torre de belem, conservas reais, royal sardine tin, portugal history art, vintage engraving, lisbon monument, iphone 18 pro max, samsung galaxy s26, tough phone case, archival travel case, architecture lover, portuguese empire</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="54" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>belem tower phone case, maritime cannery label case, vintage lisbon fortress case, royal conservas case, portugal history case</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Sardinha com Pimentos Grilled Pepper Sardine Fest Tough Case</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104806-1f1c6f39-2bce-65d6-a928-4eb37dd39630.png</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Sizzling Santos Populares street festival celebration featuring charred grilled sardines served over rustic broa cornbread with charred red and green bell peppers and summer festival garland. Durable Tough Case.</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-008</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>sardinha com pimentos, grilled sardines, santos populares, festa de lisboa, portuguese food art, sardine festival, broa cornbread, iphone 18 pro max, samsung galaxy s26, tough phone case, foodie phone case, portugal summer fest, lisbon street food</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="54" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>grilled pepper sardine case, santos populares phone case, sardinha com pimentos case, rustic food phone case, lisbon fest case</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Madeira Island Exotic Passion Fruit Sardine Tough Case</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104850-1f1c6f3a-d0c9-6972-917c-c6926db4fc70.png</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Botanical Art Nouveau vintage sardine tin label adorned with exotic Madeira passion fruit blossoms, lush banana leaves, and rugged Atlantic volcanic cliffs. Protective dual-layer Tough Case.</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-009</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>madeira island case, passion fruit tin, botanical art nouveau, tropical sardine, portugal islands, madeira flower fest, atlantic island art, iphone 18 pro max, samsung galaxy s26, tough phone case, funchal souvenir, exotic botanical, volcanic cliffs</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="54" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>madeira island phone case, passion fruit sardine case, botanical art nouveau case, tropical island phone case, exotic fruit case</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Cascais Riviera Sunbather Sardine Picnic Tough Case</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>https://d123s6f1z9g2wk.cloudfront.net/files/2026/10/20261013104935-1f1c6f3c-79c2-680c-9a78-a6efca640832.png</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Phone Cases</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Phone Cases</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Chic 1950s Mid-Century French-Portuguese Riviera gouache featuring cat-eye sunglasses, striped beach cabana umbrella, and a golden sardine tin on a sun-drenched Cascais sandy beach towel. Dual-layer Tough Case.</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.etsy.com/shop/CraftCasesStudio?utm_source=pinterest&amp;utm_medium=social&amp;utm_campaign=case-sardpt-010</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>cascais riviera, beach picnic case, retro sunbather, mid century gouache, portugal beach case, coastal summer tin, vintage 1950s resort, iphone 18 pro max, samsung galaxy s26, tough phone case, summer vacation gift, estoril coast, sandy beach picnic</t>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/shop/CraftCasesStudio</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>cascais riviera picnic case, 1950s gouache phone case, retro sunglasses beach case, luxury coastal vacation case, beach picnic case</t>
         </is>
       </c>
     </row>

</xml_diff>